<commit_message>
HOIpTP, ICpUEfEBE, NBICP, DRC, GHESS, IiCFdtTI, PMCCS, PMCRS, PMGBSA, RAF (set to 1), RQSD, PEAAC, PERAC (fix multipliers), MPoEFUbVT, RZSPbS, TTS, VTQaZ: extend all to 2070
</commit_message>
<xml_diff>
--- a/InputData/elec/DRC/Demand Response Capacity.xlsx
+++ b/InputData/elec/DRC/Demand Response Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28507"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anaxolt/Google Drive/2021/D.Development/TARGET_eps-us-3.2.1/InputData/elec/DRC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\elec\DRC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{EAF18D30-C872-8641-B28C-E82493455792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85781D6E-DF9F-47DE-9867-BAA8E93E065C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0FABC8-E2D3-43E6-A08C-2D1399C1AE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="500" windowWidth="23960" windowHeight="12280" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,6 @@
     <sheet name="DRC-PADRC" sheetId="2" r:id="rId5"/>
     <sheet name="DRC-ADRHpDRE" sheetId="7" r:id="rId6"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId7"/>
-  </externalReferences>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -191,10 +188,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000000"/>
-  </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -230,12 +224,13 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Consolas"/>
-      <charset val="1"/>
+      <family val="3"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -266,7 +261,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -277,22 +272,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -314,19 +310,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Data and Calculations"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -617,32 +600,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="107.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -650,98 +633,98 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" s="2">
         <v>2019</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -759,19 +742,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AH22"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
     </row>
-    <row r="2" spans="1:34">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2019</v>
       </c>
@@ -779,7 +762,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="3" spans="1:34">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>59000</v>
       </c>
@@ -787,12 +770,12 @@
         <v>198000</v>
       </c>
     </row>
-    <row r="5" spans="1:34" s="6" customFormat="1">
+    <row r="5" spans="1:34" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:34">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -893,7 +876,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="7" spans="1:34">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -995,44 +978,44 @@
       </c>
       <c r="AH7" s="7"/>
     </row>
-    <row r="11" spans="1:34">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
     </row>
-    <row r="13" spans="1:34">
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:34">
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:34">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>4</v>
       </c>
@@ -1046,547 +1029,548 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE2C662D-3E4B-D847-BD9D-5DB361B9A6C7}">
   <dimension ref="A1:AM6"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" customWidth="1"/>
-    <col min="2" max="13" width="9.140625"/>
-    <col min="14" max="14" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="13" width="9.140625" style="15"/>
+    <col min="14" max="14" width="16.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9" style="15" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9" style="15" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.85546875" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C1">
+      <c r="C1" s="15">
         <v>2014</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="15">
         <v>2015</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="15">
         <v>2016</v>
       </c>
-      <c r="F1">
+      <c r="F1" s="15">
         <v>2017</v>
       </c>
-      <c r="G1">
+      <c r="G1" s="15">
         <v>2018</v>
       </c>
-      <c r="H1">
+      <c r="H1" s="15">
         <v>2019</v>
       </c>
-      <c r="I1">
+      <c r="I1" s="15">
         <v>2020</v>
       </c>
-      <c r="J1">
+      <c r="J1" s="15">
         <v>2021</v>
       </c>
-      <c r="K1">
+      <c r="K1" s="15">
         <v>2022</v>
       </c>
-      <c r="L1">
+      <c r="L1" s="15">
         <v>2023</v>
       </c>
-      <c r="M1">
+      <c r="M1" s="15">
         <v>2024</v>
       </c>
-      <c r="N1">
+      <c r="N1" s="15">
         <v>2025</v>
       </c>
-      <c r="O1">
+      <c r="O1" s="15">
         <v>2026</v>
       </c>
-      <c r="P1">
+      <c r="P1" s="15">
         <v>2027</v>
       </c>
-      <c r="Q1">
+      <c r="Q1" s="15">
         <v>2028</v>
       </c>
-      <c r="R1">
+      <c r="R1" s="15">
         <v>2029</v>
       </c>
-      <c r="S1">
+      <c r="S1" s="15">
         <v>2030</v>
       </c>
-      <c r="T1">
+      <c r="T1" s="15">
         <v>2031</v>
       </c>
-      <c r="U1">
+      <c r="U1" s="15">
         <v>2032</v>
       </c>
-      <c r="V1">
+      <c r="V1" s="15">
         <v>2033</v>
       </c>
-      <c r="W1">
+      <c r="W1" s="15">
         <v>2034</v>
       </c>
-      <c r="X1">
+      <c r="X1" s="15">
         <v>2035</v>
       </c>
-      <c r="Y1">
+      <c r="Y1" s="15">
         <v>2036</v>
       </c>
-      <c r="Z1">
+      <c r="Z1" s="15">
         <v>2037</v>
       </c>
-      <c r="AA1">
+      <c r="AA1" s="15">
         <v>2038</v>
       </c>
-      <c r="AB1">
+      <c r="AB1" s="15">
         <v>2039</v>
       </c>
-      <c r="AC1">
+      <c r="AC1" s="15">
         <v>2040</v>
       </c>
-      <c r="AD1">
+      <c r="AD1" s="15">
         <v>2041</v>
       </c>
-      <c r="AE1">
+      <c r="AE1" s="15">
         <v>2042</v>
       </c>
-      <c r="AF1">
+      <c r="AF1" s="15">
         <v>2043</v>
       </c>
-      <c r="AG1">
+      <c r="AG1" s="15">
         <v>2044</v>
       </c>
-      <c r="AH1">
+      <c r="AH1" s="15">
         <v>2045</v>
       </c>
-      <c r="AI1">
+      <c r="AI1" s="15">
         <v>2046</v>
       </c>
-      <c r="AJ1">
+      <c r="AJ1" s="15">
         <v>2047</v>
       </c>
-      <c r="AK1">
+      <c r="AK1" s="15">
         <v>2048</v>
       </c>
-      <c r="AL1">
+      <c r="AL1" s="15">
         <v>2049</v>
       </c>
-      <c r="AM1">
+      <c r="AM1" s="15">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:39">
-      <c r="A2" s="5"/>
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A2" s="16"/>
+      <c r="B2" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="15">
         <v>9.8636644841800333E-2</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="15">
         <v>0.1003252824664638</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="15">
         <v>0.10104496285900474</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="15">
         <v>0.10152702997943744</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="15">
         <v>0.10197979351839384</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="15">
         <v>0.10245639964773269</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="15">
         <v>0.10296756277334541</v>
       </c>
-      <c r="J2" s="9">
+      <c r="J2" s="15">
         <v>0.10340803251068771</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="15">
         <v>0.10388755191988928</v>
       </c>
-      <c r="L2" s="9">
+      <c r="L2" s="15">
         <v>0.10440602714772437</v>
       </c>
-      <c r="M2" s="9">
+      <c r="M2" s="15">
         <v>0.10496009002297045</v>
       </c>
-      <c r="N2" s="9">
+      <c r="N2" s="15">
         <v>0.10556555417442678</v>
       </c>
-      <c r="O2" s="9">
+      <c r="O2" s="15">
         <v>0.10600870488733041</v>
       </c>
-      <c r="P2" s="9">
+      <c r="P2" s="15">
         <v>0.10652912605952648</v>
       </c>
-      <c r="Q2" s="9">
+      <c r="Q2" s="15">
         <v>0.10713820378721554</v>
       </c>
-      <c r="R2" s="9">
+      <c r="R2" s="15">
         <v>0.1078432446493542</v>
       </c>
-      <c r="S2" s="9">
+      <c r="S2" s="15">
         <v>0.10864823793881466</v>
       </c>
-      <c r="T2" s="9">
+      <c r="T2" s="15">
         <v>0.10949499278959707</v>
       </c>
-      <c r="U2" s="9">
+      <c r="U2" s="15">
         <v>0.11043742468059306</v>
       </c>
-      <c r="V2" s="9">
+      <c r="V2" s="15">
         <v>0.11146883731544265</v>
       </c>
-      <c r="W2" s="9">
+      <c r="W2" s="15">
         <v>0.11257986730772145</v>
       </c>
-      <c r="X2" s="9">
+      <c r="X2" s="15">
         <v>0.11375854360098116</v>
       </c>
-      <c r="Y2" s="9">
+      <c r="Y2" s="15">
         <v>0.11500700295303776</v>
       </c>
-      <c r="Z2" s="9">
+      <c r="Z2" s="15">
         <v>0.11629345638152376</v>
       </c>
-      <c r="AA2" s="9">
+      <c r="AA2" s="15">
         <v>0.11760210049057489</v>
       </c>
-      <c r="AB2" s="9">
+      <c r="AB2" s="15">
         <v>0.11891740974492833</v>
       </c>
-      <c r="AC2" s="9">
+      <c r="AC2" s="15">
         <v>0.12022482270847104</v>
       </c>
-      <c r="AD2" s="9">
+      <c r="AD2" s="15">
         <v>0.1217335942417123</v>
       </c>
-      <c r="AE2" s="9">
+      <c r="AE2" s="15">
         <v>0.12321472992477742</v>
       </c>
-      <c r="AF2" s="9">
+      <c r="AF2" s="15">
         <v>0.12465772297340184</v>
       </c>
-      <c r="AG2" s="9">
+      <c r="AG2" s="15">
         <v>0.12605355536241392</v>
       </c>
-      <c r="AH2" s="9">
+      <c r="AH2" s="15">
         <v>0.12739430164149732</v>
       </c>
-      <c r="AI2" s="9">
+      <c r="AI2" s="15">
         <v>0.12879656057806463</v>
       </c>
-      <c r="AJ2" s="9">
+      <c r="AJ2" s="15">
         <v>0.13011576903115954</v>
       </c>
-      <c r="AK2" s="9">
+      <c r="AK2" s="15">
         <v>0.13135142612657708</v>
       </c>
-      <c r="AL2" s="9">
+      <c r="AL2" s="15">
         <v>0.13250370221109664</v>
       </c>
-      <c r="AM2" s="9">
+      <c r="AM2" s="15">
         <v>0.13357320132464462</v>
       </c>
     </row>
-    <row r="3" spans="1:39">
-      <c r="B3" t="s">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="B3" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="9">
-        <v>0</v>
-      </c>
-      <c r="D3" s="9">
-        <v>0</v>
-      </c>
-      <c r="E3" s="9">
-        <v>0</v>
-      </c>
-      <c r="F3" s="9">
-        <v>0</v>
-      </c>
-      <c r="G3" s="9">
-        <v>0</v>
-      </c>
-      <c r="H3" s="9">
-        <v>0</v>
-      </c>
-      <c r="I3" s="9">
-        <v>0</v>
-      </c>
-      <c r="J3" s="9">
-        <v>0</v>
-      </c>
-      <c r="K3" s="9">
-        <v>0</v>
-      </c>
-      <c r="L3" s="9">
-        <v>0</v>
-      </c>
-      <c r="M3" s="9">
-        <v>0</v>
-      </c>
-      <c r="N3" s="9">
+      <c r="C3" s="15">
+        <v>0</v>
+      </c>
+      <c r="D3" s="15">
+        <v>0</v>
+      </c>
+      <c r="E3" s="15">
+        <v>0</v>
+      </c>
+      <c r="F3" s="15">
+        <v>0</v>
+      </c>
+      <c r="G3" s="15">
+        <v>0</v>
+      </c>
+      <c r="H3" s="15">
+        <v>0</v>
+      </c>
+      <c r="I3" s="15">
+        <v>0</v>
+      </c>
+      <c r="J3" s="15">
+        <v>0</v>
+      </c>
+      <c r="K3" s="15">
+        <v>0</v>
+      </c>
+      <c r="L3" s="15">
+        <v>0</v>
+      </c>
+      <c r="M3" s="15">
+        <v>0</v>
+      </c>
+      <c r="N3" s="15">
         <f t="shared" ref="N3:W3" si="0">(($X3-$M3)/($X1-$M1))*(N1-$M1)+$M3</f>
         <v>9.0909090909090912E-2</v>
       </c>
-      <c r="O3" s="9">
+      <c r="O3" s="15">
         <f t="shared" si="0"/>
         <v>0.18181818181818182</v>
       </c>
-      <c r="P3" s="9">
-        <f t="shared" si="0"/>
+      <c r="P3" s="15">
+        <f>(($X3-$M3)/($X1-$M1))*(P1-$M1)+$M3</f>
         <v>0.27272727272727271</v>
       </c>
-      <c r="Q3" s="9">
+      <c r="Q3" s="15">
         <f t="shared" si="0"/>
         <v>0.36363636363636365</v>
       </c>
-      <c r="R3" s="9">
+      <c r="R3" s="15">
         <f t="shared" si="0"/>
         <v>0.45454545454545459</v>
       </c>
-      <c r="S3" s="9">
+      <c r="S3" s="15">
         <f t="shared" si="0"/>
         <v>0.54545454545454541</v>
       </c>
-      <c r="T3" s="9">
+      <c r="T3" s="15">
         <f t="shared" si="0"/>
         <v>0.63636363636363635</v>
       </c>
-      <c r="U3" s="9">
+      <c r="U3" s="15">
         <f t="shared" si="0"/>
         <v>0.72727272727272729</v>
       </c>
-      <c r="V3" s="9">
+      <c r="V3" s="15">
         <f t="shared" si="0"/>
         <v>0.81818181818181823</v>
       </c>
-      <c r="W3" s="9">
+      <c r="W3" s="15">
         <f t="shared" si="0"/>
         <v>0.90909090909090917</v>
       </c>
-      <c r="X3" s="9">
+      <c r="X3" s="15">
         <v>1</v>
       </c>
-      <c r="Y3" s="9">
+      <c r="Y3" s="15">
         <v>1</v>
       </c>
-      <c r="Z3" s="9">
+      <c r="Z3" s="15">
         <v>1</v>
       </c>
-      <c r="AA3" s="9">
+      <c r="AA3" s="15">
         <v>1</v>
       </c>
-      <c r="AB3" s="9">
+      <c r="AB3" s="15">
         <v>1</v>
       </c>
-      <c r="AC3" s="9">
+      <c r="AC3" s="15">
         <v>1</v>
       </c>
-      <c r="AD3" s="9">
+      <c r="AD3" s="15">
         <v>1</v>
       </c>
-      <c r="AE3" s="9">
+      <c r="AE3" s="15">
         <v>1</v>
       </c>
-      <c r="AF3" s="9">
+      <c r="AF3" s="15">
         <v>1</v>
       </c>
-      <c r="AG3" s="9">
+      <c r="AG3" s="15">
         <v>1</v>
       </c>
-      <c r="AH3" s="9">
+      <c r="AH3" s="15">
         <v>1</v>
       </c>
-      <c r="AI3" s="9">
+      <c r="AI3" s="15">
         <v>1</v>
       </c>
-      <c r="AJ3" s="9">
+      <c r="AJ3" s="15">
         <v>1</v>
       </c>
-      <c r="AK3" s="9">
+      <c r="AK3" s="15">
         <v>1</v>
       </c>
-      <c r="AL3" s="9">
+      <c r="AL3" s="15">
         <v>1</v>
       </c>
-      <c r="AM3" s="9">
+      <c r="AM3" s="15">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:39">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A4" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="15">
         <f t="shared" ref="C4:AM4" si="1">C2*C3</f>
         <v>0</v>
       </c>
-      <c r="D4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="L4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M4" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N4" s="9">
+      <c r="D4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="M4" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N4" s="15">
         <f t="shared" si="1"/>
         <v>9.5968685613115265E-3</v>
       </c>
-      <c r="O4" s="9">
+      <c r="O4" s="15">
         <f t="shared" si="1"/>
         <v>1.9274309979514622E-2</v>
       </c>
-      <c r="P4" s="9">
-        <f t="shared" si="1"/>
+      <c r="P4" s="15">
+        <f>P2*P3</f>
         <v>2.9053398016234494E-2</v>
       </c>
-      <c r="Q4" s="9">
+      <c r="Q4" s="15">
         <f t="shared" si="1"/>
         <v>3.8959346831714745E-2</v>
       </c>
-      <c r="R4" s="9">
+      <c r="R4" s="15">
         <f t="shared" si="1"/>
         <v>4.9019656658797366E-2</v>
       </c>
-      <c r="S4" s="9">
+      <c r="S4" s="15">
         <f t="shared" si="1"/>
         <v>5.9262675239353448E-2</v>
       </c>
-      <c r="T4" s="9">
+      <c r="T4" s="15">
         <f t="shared" si="1"/>
         <v>6.9678631775198133E-2</v>
       </c>
-      <c r="U4" s="9">
+      <c r="U4" s="15">
         <f t="shared" si="1"/>
         <v>8.0318127040431314E-2</v>
       </c>
-      <c r="V4" s="9">
+      <c r="V4" s="15">
         <f t="shared" si="1"/>
         <v>9.1201775985362166E-2</v>
       </c>
-      <c r="W4" s="9">
+      <c r="W4" s="15">
         <f t="shared" si="1"/>
         <v>0.10234533391611042</v>
       </c>
-      <c r="X4" s="9">
+      <c r="X4" s="15">
         <f t="shared" si="1"/>
         <v>0.11375854360098116</v>
       </c>
-      <c r="Y4" s="9">
+      <c r="Y4" s="15">
         <f t="shared" si="1"/>
         <v>0.11500700295303776</v>
       </c>
-      <c r="Z4" s="9">
+      <c r="Z4" s="15">
         <f t="shared" si="1"/>
         <v>0.11629345638152376</v>
       </c>
-      <c r="AA4" s="9">
+      <c r="AA4" s="15">
         <f t="shared" si="1"/>
         <v>0.11760210049057489</v>
       </c>
-      <c r="AB4" s="9">
+      <c r="AB4" s="15">
         <f t="shared" si="1"/>
         <v>0.11891740974492833</v>
       </c>
-      <c r="AC4" s="9">
+      <c r="AC4" s="15">
         <f t="shared" si="1"/>
         <v>0.12022482270847104</v>
       </c>
-      <c r="AD4" s="9">
+      <c r="AD4" s="15">
         <f t="shared" si="1"/>
         <v>0.1217335942417123</v>
       </c>
-      <c r="AE4" s="9">
+      <c r="AE4" s="15">
         <f t="shared" si="1"/>
         <v>0.12321472992477742</v>
       </c>
-      <c r="AF4" s="9">
+      <c r="AF4" s="15">
         <f t="shared" si="1"/>
         <v>0.12465772297340184</v>
       </c>
-      <c r="AG4" s="9">
+      <c r="AG4" s="15">
         <f t="shared" si="1"/>
         <v>0.12605355536241392</v>
       </c>
-      <c r="AH4" s="9">
+      <c r="AH4" s="15">
         <f t="shared" si="1"/>
         <v>0.12739430164149732</v>
       </c>
-      <c r="AI4" s="9">
+      <c r="AI4" s="15">
         <f t="shared" si="1"/>
         <v>0.12879656057806463</v>
       </c>
-      <c r="AJ4" s="9">
+      <c r="AJ4" s="15">
         <f t="shared" si="1"/>
         <v>0.13011576903115954</v>
       </c>
-      <c r="AK4" s="9">
+      <c r="AK4" s="15">
         <f t="shared" si="1"/>
         <v>0.13135142612657708</v>
       </c>
-      <c r="AL4" s="9">
+      <c r="AL4" s="15">
         <f t="shared" si="1"/>
         <v>0.13250370221109664</v>
       </c>
-      <c r="AM4" s="9">
+      <c r="AM4" s="15">
         <f t="shared" si="1"/>
         <v>0.13357320132464462</v>
       </c>
     </row>
-    <row r="5" spans="1:39">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:39">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1601,13 +1585,13 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AH16"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:BD16"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -1710,8 +1694,68 @@
       <c r="AH1">
         <v>2050</v>
       </c>
-    </row>
-    <row r="2" spans="1:34">
+      <c r="AI1">
+        <v>2051</v>
+      </c>
+      <c r="AJ1">
+        <v>2052</v>
+      </c>
+      <c r="AK1">
+        <v>2053</v>
+      </c>
+      <c r="AL1">
+        <v>2054</v>
+      </c>
+      <c r="AM1">
+        <v>2055</v>
+      </c>
+      <c r="AN1">
+        <v>2056</v>
+      </c>
+      <c r="AO1">
+        <v>2057</v>
+      </c>
+      <c r="AP1">
+        <v>2058</v>
+      </c>
+      <c r="AQ1">
+        <v>2059</v>
+      </c>
+      <c r="AR1">
+        <v>2060</v>
+      </c>
+      <c r="AS1">
+        <v>2061</v>
+      </c>
+      <c r="AT1">
+        <v>2062</v>
+      </c>
+      <c r="AU1">
+        <v>2063</v>
+      </c>
+      <c r="AV1">
+        <v>2064</v>
+      </c>
+      <c r="AW1">
+        <v>2065</v>
+      </c>
+      <c r="AX1">
+        <v>2066</v>
+      </c>
+      <c r="AY1">
+        <v>2067</v>
+      </c>
+      <c r="AZ1">
+        <v>2068</v>
+      </c>
+      <c r="BA1">
+        <v>2069</v>
+      </c>
+      <c r="BB1">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="2" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>42</v>
       </c>
@@ -1719,7 +1763,7 @@
         <f>C2</f>
         <v>0</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="10">
         <f>'Data and Calculations'!A3*'Scaling Factors'!H4</f>
         <v>0</v>
       </c>
@@ -1847,9 +1891,91 @@
         <f>('Data and Calculations'!$A3)*('Data and Calculations'!AG7/'Data and Calculations'!$B$7)*'Scaling Factors'!AM4</f>
         <v>9665.2501222709798</v>
       </c>
-    </row>
-    <row r="16" spans="1:34">
-      <c r="E16" s="12"/>
+      <c r="AI2" s="4">
+        <f>AH2</f>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AJ2" s="4">
+        <f t="shared" ref="AJ2:BB2" si="0">AI2</f>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AK2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AL2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AM2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AN2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AO2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AP2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AQ2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AR2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AS2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AT2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AU2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AV2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AW2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AX2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AY2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="AZ2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="BA2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="BB2" s="4">
+        <f t="shared" si="0"/>
+        <v>9665.2501222709798</v>
+      </c>
+      <c r="BC2" s="4"/>
+      <c r="BD2" s="4"/>
+    </row>
+    <row r="16" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="E16" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1861,13 +1987,13 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:BB2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -1970,16 +2096,76 @@
       <c r="AH1">
         <v>2050</v>
       </c>
-    </row>
-    <row r="2" spans="1:34">
-      <c r="A2" s="17" t="s">
+      <c r="AI1">
+        <v>2051</v>
+      </c>
+      <c r="AJ1">
+        <v>2052</v>
+      </c>
+      <c r="AK1">
+        <v>2053</v>
+      </c>
+      <c r="AL1">
+        <v>2054</v>
+      </c>
+      <c r="AM1">
+        <v>2055</v>
+      </c>
+      <c r="AN1">
+        <v>2056</v>
+      </c>
+      <c r="AO1">
+        <v>2057</v>
+      </c>
+      <c r="AP1">
+        <v>2058</v>
+      </c>
+      <c r="AQ1">
+        <v>2059</v>
+      </c>
+      <c r="AR1">
+        <v>2060</v>
+      </c>
+      <c r="AS1">
+        <v>2061</v>
+      </c>
+      <c r="AT1">
+        <v>2062</v>
+      </c>
+      <c r="AU1">
+        <v>2063</v>
+      </c>
+      <c r="AV1">
+        <v>2064</v>
+      </c>
+      <c r="AW1">
+        <v>2065</v>
+      </c>
+      <c r="AX1">
+        <v>2066</v>
+      </c>
+      <c r="AY1">
+        <v>2067</v>
+      </c>
+      <c r="AZ1">
+        <v>2068</v>
+      </c>
+      <c r="BA1">
+        <v>2069</v>
+      </c>
+      <c r="BB1">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="2" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B2" s="4">
         <f>C2*'Scaling Factors'!G2</f>
         <v>410.56326324847817</v>
       </c>
-      <c r="C2" s="15">
+      <c r="C2" s="12">
         <f>'Data and Calculations'!A3*'Scaling Factors'!H2-'DRC-BDRC'!C1</f>
         <v>4025.9275792162289</v>
       </c>
@@ -2105,6 +2291,86 @@
       </c>
       <c r="AH2" s="4">
         <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AH1)*'Scaling Factors'!AM2-'DRC-BDRC'!AH2</f>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AI2" s="4">
+        <f>AH2</f>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AJ2" s="4">
+        <f t="shared" ref="AJ2:BB2" si="0">AI2</f>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AK2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AL2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AM2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AN2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AO2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AP2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AQ2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AR2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AS2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AT2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AU2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AV2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AW2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AX2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AY2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="AZ2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="BA2" s="4">
+        <f t="shared" si="0"/>
+        <v>50539.834620237118</v>
+      </c>
+      <c r="BB2" s="4">
+        <f t="shared" si="0"/>
         <v>50539.834620237118</v>
       </c>
     </row>
@@ -2119,21 +2385,21 @@
     <tabColor rgb="FF1F497D"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="4">
         <f>ROUND('Data and Calculations'!A22,0)</f>
         <v>4</v>
       </c>
@@ -2144,21 +2410,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -2302,14 +2553,52 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD124F93-4C1F-4E6F-9FF6-BBDFC587A76D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EC3B175-1A50-44DD-A6FF-610DA475B8B5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC1EE97F-BEF3-4E27-B60F-7AF2FDABE2B4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC1EE97F-BEF3-4E27-B60F-7AF2FDABE2B4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EC3B175-1A50-44DD-A6FF-610DA475B8B5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD124F93-4C1F-4E6F-9FF6-BBDFC587A76D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>